<commit_message>
Add 15 MT_CLIENT_DB data quality queries; add schema explorer and query generator scripts
</commit_message>
<xml_diff>
--- a/input/input_queries.xlsx
+++ b/input/input_queries.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Queries" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,10 +55,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -425,83 +428,335 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>query</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SELECT customer_id, name FROM customers WHERE age IS NULL</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Q01 - Customers with NULL name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    customer_id,
+    account_type,
+    region,
+    join_date
+FROM CUSTOMERS
+WHERE customer_name IS NULL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SELECT id, name FROM customers</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Q02 - Transactions with NULL amount</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    transaction_id,
+    customer_id,
+    tx_date,
+    tx_type,
+    status
+FROM TRANSACTIONS
+WHERE amount IS NULL</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>SELECT id FROM orders WHERE amount &lt;= 0 AND status = 'PENDING'</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Q03 - Transactions with negative amount</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    transaction_id,
+    customer_id,
+    tx_date,
+    tx_type,
+    amount,
+    status
+FROM TRANSACTIONS
+WHERE amount &lt; 0</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SELECT a.id FROM customers a LEFT JOIN addresses b ON a.id = b.customer_id WHERE a.status = 'ACTIVE' AND b.country = 'US'</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Q04 - Transactions with invalid status</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    transaction_id,
+    customer_id,
+    tx_date,
+    amount,
+    status
+FROM TRANSACTIONS
+WHERE status NOT IN ('COMPLETED', 'PENDING', 'FAILED', 'REVERSED')</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>SELECT a.id FROM customers a WHERE a.id IN (SELECT customer_id FROM orders WHERE status = 'ACTIVE')</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Q05 - Customers with unrecognised risk rating</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    customer_id,
+    customer_name,
+    account_type,
+    risk_rating
+FROM CUSTOMERS
+WHERE risk_rating NOT IN ('LOW', 'MEDIUM', 'HIGH')</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>WITH customer_data AS (    SELECT * FROM customers WHERE status = 'ACTIVE') SELECT * FROM customer_data WHERE age IS NULL</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Q06 - Orphaned transactions (no matching customer)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    t.transaction_id,
+    t.customer_id,
+    t.tx_date,
+    t.amount,
+    t.status
+FROM TRANSACTIONS t
+LEFT JOIN CUSTOMERS c
+    ON t.customer_id = c.customer_id
+WHERE c.customer_id IS NULL</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>SELECT c.id FROM customers c WHERE EXISTS (    SELECT 1 FROM orders o     WHERE o.customer_id = c.id AND o.status = 'CANCELLED')</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Q07 - Transactions referencing unknown product</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    t.transaction_id,
+    t.customer_id,
+    t.product_id,
+    t.amount,
+    t.tx_date
+FROM TRANSACTIONS t
+LEFT JOIN PRODUCTS p
+    ON t.product_id = p.product_id
+WHERE p.product_id IS NULL</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SELECT id FROM transactions WHERE CASE WHEN amount &gt; 0 THEN 'CREDIT' ELSE 'DEBIT' END = 'DEBIT'</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Q08 - Account summary records with no matching customer</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    a.account_id,
+    a.customer_id,
+    a.current_balance,
+    a.currency,
+    a.last_updated
+FROM ACCOUNT_SUMMARY a
+LEFT JOIN CUSTOMERS c
+    ON a.customer_id = c.customer_id
+WHERE c.customer_id IS NULL</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SELECT id FROM events WHERE DATEDIFF('day', created_at, CURRENT_DATE()) &gt; 30</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Q09 - Customers with no transaction history</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    customer_id,
+    customer_name,
+    account_type,
+    risk_rating,
+    join_date
+FROM CUSTOMERS
+WHERE customer_id NOT IN (
+    SELECT DISTINCT customer_id
+    FROM TRANSACTIONS
+    WHERE customer_id IS NOT NULL
+)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SELECT a.id FROM customers a WHERE a.region_id IN (    SELECT region_id FROM regions     WHERE country_id IN (        SELECT country_id FROM countries WHERE iso_code = 'US'    ))</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Q10 - Accounts with at least one FAILED transaction</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    a.account_id,
+    a.customer_id,
+    a.current_balance,
+    a.currency
+FROM ACCOUNT_SUMMARY a
+WHERE EXISTS (
+    SELECT 1
+    FROM TRANSACTIONS t
+    WHERE t.customer_id = a.customer_id
+      AND t.status = 'FAILED'
+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Q11 - Transactions with future TX_DATE</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    transaction_id,
+    customer_id,
+    tx_date,
+    amount,
+    status
+FROM TRANSACTIONS
+WHERE tx_date &gt; CURRENT_DATE()</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Q12 - Accounts with negative current balance</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    account_id,
+    customer_id,
+    current_balance,
+    currency,
+    last_updated
+FROM ACCOUNT_SUMMARY
+WHERE current_balance &lt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Q13 - Products with NULL or zero minimum balance</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    product_id,
+    product_name,
+    category,
+    interest_rate_pct,
+    min_balance
+FROM PRODUCTS
+WHERE min_balance IS NULL
+   OR min_balance &lt;= 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Q14 - High-risk customers with negative account balances (CTE)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>WITH high_risk_customers AS (
+    SELECT
+        customer_id,
+        customer_name,
+        risk_rating
+    FROM CUSTOMERS
+    WHERE risk_rating = 'HIGH'
+)
+SELECT
+    a.account_id,
+    h.customer_name,
+    h.risk_rating,
+    a.current_balance,
+    a.currency
+FROM ACCOUNT_SUMMARY a
+INNER JOIN high_risk_customers h
+    ON a.customer_id = h.customer_id
+WHERE a.current_balance &lt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Q15 - Transactions missing critical fields (tx_type, status, or branch_code)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SELECT
+    transaction_id,
+    customer_id,
+    product_id,
+    tx_date,
+    tx_type,
+    status,
+    branch_code
+FROM TRANSACTIONS
+WHERE tx_type IS NULL
+   OR status IS NULL
+   OR branch_code IS NULL</t>
         </is>
       </c>
     </row>

</xml_diff>